<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.001-05 Le camion sous le robinet
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.001-05.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.001-05.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin, robinet, torchon à carreaux, plaid</t>
+          <t>jardin, robinet, torchon à carreaux, plaid, camion de bois</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amir, Sarah, maman</t>
+          <t>Amir, Sarah, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut laver le camion de bois pour un voyage jusqu'au plaid. Sarah est plus grande, le robinet est haut. Ils lavent ensemble. Le camion brille et roule.</t>
+          <t>Le robinet du jardin fait tic. Une goutte tient. Sur le métal, un éclat de robinet brille. Amir veut laver le camion de bois maintenant, pour un voyage jusqu'au plaid. Il invite Sarah. Ils ne veulent pas la même chose : les roues contre l'eau. Le camion glisse, l'éclat saute. Ils refusent de foncer, écoutent le tic. Sarah tient le toit, Amir frotte les roues. Merci vécu. Le camion file vers le plaid. Ils le prennent des deux bords. L'éclat de robinet tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le torchon à carreaux sent le savon. Il sèche sur la pierre. Le petit camion de bois a de la poussière. Les carreaux du jardin sont chauds. Le robinet goutte, tout lent. Une coccinelle marche sur une feuille. Tu as vu le torchon, Amir ? Oui, maman. Il sent le propre. Oui. Je veux laver le camion. Pour un voyage, après ? Oui. En ce moment, Amir prend le camion. Le bois est sec, un peu rêche. Sarah arrive avec le seau. Sarah est plus grande. Amir est plus petit. Ils ont des tailles différentes. Tu viens ? On lave le camion. Oui. Maman ouvre le robinet, tout doux. L'eau est tiède. Elle brille sur les carreaux. Je n'atteins pas. Sarah tient le camion. Toi, tu frottes les roues. Vous jouez ensemble. On peut jouer ensemble. Sarah tient le toit sous l'eau. Amir frotte les roues. Le torchon est mouillé, maintenant. Ça mousse un peu ! Oui. Le toit brille. Les roues aussi. Une goutte tombe sur un carreau. Elle fait un petit chemin. On laisse la coccinelle ? Oui. Le camion n'a plus de poussière. Le bois est foncé, tout propre. Une goutte reste sur le capot. Elle brille. Oui. Le bois a bu un peu.</t>
+          <t>Le robinet du jardin fait tic. Une goutte tient, ronde. Sur le métal, un éclat de robinet brille. Amir connaît ce jardin, après le soleil. Un détail paraît nouveau, sur le bec. Tu le vois, Amir ? Oui, maman. Il brille. C'est l'eau, sur le métal. Le torchon à carreaux sèche sur la pierre. Il sent le savon. Un petit camion de bois attend. Le bois a de la poussière. Un plaid tiède repose près des tomates. Je veux laver le camion, maintenant ! Pour un voyage, après ? Oui. Jusqu'au plaid. Tes mains, Amir ? Elles sont prêtes. Sarah arrive près de la pierre. Tu viens ? On lave le camion. Oui. En ce moment, Amir prend le camion. Le bois est sec, un peu rêche. Sarah pose une main sur le toit. Amir pose une main sur une roue. Moi, je mets de l'eau. Moi, les roues. Un peu d'eau ? Oui, papa. Un filet tiède tombe sur la pierre. Amir tire vers les roues. Sarah tire vers l'eau. Les roues, Sarah ! L'eau d'abord ! Le camion glisse. Il tape la pierre. L'eau gicle sur le torchon. Oh. Il est parti. L'éclat de robinet saute. Une goutte le cache. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux le camion propre ? Oui, papa. Sarah, tu le tiens ? Oui, maman. Tu tiens ma manche, Amir ? Oui. Amir veut recommencer tout de suite. Ses doigts foncent vers le bois. Je le veux maintenant !</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le torchon à carreaux sent le savon. Il sèche sur la pierre. Le petit camion de bois a de la poussière. Les carreaux du jardin sont chauds. Le robinet goutte, tout lent. Une coccinelle marche sur une feuille. Tu as vu le torchon, Amir ? Oui, maman. Il sent le propre. Oui. Je veux laver le camion. Pour un voyage, après ? Oui. En ce moment, Amir prend le camion. Le bois est sec, un peu rêche. Sarah arrive avec le seau. Sarah est plus grande. Amir est plus petit. Ils ont des tailles différentes. Tu viens ? On lave le camion. Oui. Maman ouvre le robinet, tout doux. L'eau est tiède. Elle brille sur les carreaux. Je n'atteins pas. Sarah tient le camion. Toi, tu frottes les roues. Vous jouez ensemble. On peut jouer ensemble. Sarah tient le toit sous l'eau. Amir frotte les roues. Le torchon est mouillé, maintenant. Ça mousse un peu ! Oui. Le toit brille. Les roues aussi. Une goutte tombe sur un carreau. Elle fait un petit chemin. On laisse la coccinelle ? Oui. Le camion n'a plus de poussière. Le bois est foncé, tout propre. Une goutte reste sur le capot. Elle brille. Oui. Le bois a bu un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le robinet du jardin fait tic. Une goutte tient, ronde. Sur le métal, un &lt;emphasis level="moderate"&gt;éclat de robinet&lt;/emphasis&gt; brille. Amir connaît ce jardin, après le soleil. Un détail paraît nouveau, sur le bec. Tu le vois, Amir ? Oui, maman. Il brille. C'est l'eau, sur le métal. Le torchon à carreaux sèche sur la pierre. Il sent le savon. Un petit camion de bois attend. Le bois a de la poussière. Un plaid tiède repose près des tomates. Je veux laver le camion, maintenant ! Pour un voyage, après ? Oui. Jusqu'au plaid. Tes mains, Amir ? Elles sont prêtes. Sarah arrive près de la pierre. Tu viens ? On lave le camion. Oui. En ce moment, Amir prend le camion. Le bois est sec, un peu rêche. Sarah pose une main sur le toit. Amir pose une main sur une roue. Moi, je mets de l'eau. Moi, les roues. Un peu d'eau ? Oui, papa. Un filet tiède tombe sur la pierre. Amir tire vers les roues. Sarah tire vers l'eau. Les roues, Sarah ! L'eau d'abord ! Le camion glisse. Il tape la pierre. L'eau gicle sur le torchon. Oh. Il est parti. L'éclat de robinet saute. Une goutte le cache. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux le camion propre ? Oui, papa. Sarah, tu le tiens ? Oui, maman. Tu tiens ma manche, Amir ? Oui. Amir veut recommencer tout de suite. Ses doigts foncent vers le bois. Je le veux maintenant !&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;C'est l'après-midi. Achille est dans le jardin. Maman est près des fleurs. Diane arrive avec un seau. Diane est plus grande. Achille est plus petit. Ils ont des &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. Achille veut du sable. Il prend une petite pelle. Il va vers Diane. Il l'invite. Achille dit : viens jouer. Diane dit : oui. Ils jouent ensemble près du bac. Diane porte un gros seau. Achille porte un petit seau. Les tailles différentes restent là. Ils remplissent le bac. Maman dit : vous jouez ensemble. Achille donne une pelle. Diane donne un moule. Ils font un gâteau de sable. Petit ou grand, on joue ensemble. Maman dit : vous avez des tailles différentes. Et vous jouez ensemble.&lt;/slow&gt; [pause]</t>
+          <t>Le robinet du jardin fait tic. Une goutte tient, ronde. Sur le métal, un &lt;emphasis&gt;éclat de robinet&lt;/emphasis&gt; brille. Amir connaît ce jardin, après le soleil. Un détail paraît nouveau, sur le bec. Tu le vois, Amir ? Oui, maman. Il brille. C'est l'eau, sur le métal. Le torchon à carreaux sèche sur la pierre. Il sent le savon. Un petit camion de bois attend. Le bois a de la poussière. Un plaid tiède repose près des tomates. Je veux laver le camion, maintenant ! Pour un voyage, après ? Oui. Jusqu'au plaid. Tes mains, Amir ? Elles sont prêtes. Sarah arrive près de la pierre. Tu viens ? On lave le camion. Oui. En ce moment, Amir prend le camion. Le bois est sec, un peu rêche. Sarah pose une main sur le toit. Amir pose une main sur une roue. Moi, je mets de l'eau. Moi, les roues. Un peu d'eau ? Oui, papa. Un filet tiède tombe sur la pierre. Amir tire vers les roues. Sarah tire vers l'eau. Les roues, Sarah ! L'eau d'abord ! Le camion glisse. Il tape la pierre. L'eau gicle sur le torchon. Oh. Il est parti. L'éclat de robinet saute. Une goutte le cache. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux le camion propre ? Oui, papa. Sarah, tu le tiens ? Oui, maman. Tu tiens ma manche, Amir ? Oui. Amir veut recommencer tout de suite. Ses doigts foncent vers le bois. Je le veux maintenant ! [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>éclat de robinet</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,58 +1324,76 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_invite_sarah_mais_ils_ne_veulent_pas_la_meme_chose; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le torchon à carreaux sent le savon.
-narrateur|Il sèche sur la pierre.
-narrateur|Le petit camion de bois a de la poussière.
-narrateur|Les carreaux du jardin sont chauds.
-narrateur|Le robinet goutte, tout lent.
-narrateur|Une coccinelle marche sur une feuille.
-maman|Tu as vu le torchon, Amir ?
+          <t>narrateur|Le robinet du jardin fait tic.
+narrateur|Une goutte tient, ronde.
+narrateur|Sur le métal, un éclat de robinet brille.
+narrateur|Amir connaît ce jardin, après le soleil.
+narrateur|Un détail paraît nouveau, sur le bec.
+maman|Tu le vois, Amir ?
 enfant-m|Oui, maman.
-enfant-m|Il sent le propre.
-maman|Oui.
-enfant-m|Je veux laver le camion.
+enfant-m|Il brille.
+papa|C'est l'eau, sur le métal.
+narrateur|Le torchon à carreaux sèche sur la pierre.
+narrateur|Il sent le savon.
+narrateur|Un petit camion de bois attend.
+narrateur|Le bois a de la poussière.
+narrateur|Un plaid tiède repose près des tomates.
+enfant-m|Je veux laver le camion, maintenant !
 maman|Pour un voyage, après ?
 enfant-m|Oui.
+enfant-m|Jusqu'au plaid.
+papa|Tes mains, Amir ?
+enfant-m|Elles sont prêtes.
+narrateur|Sarah arrive près de la pierre.
+enfant-m|Tu viens ?
+enfant-m|On lave le camion.
+enfant-f|Oui.
 narrateur|En ce moment, Amir prend le camion.
 narrateur|Le bois est sec, un peu rêche.
-narrateur|Sarah arrive avec le seau.
-narrateur|Sarah est plus grande.
-narrateur|Amir est plus petit.
-narrateur|Ils ont des tailles différentes.
-enfant-m|Tu viens ?
-enfant-m|On lave le camion.
-copine|Oui.
-narrateur|Maman ouvre le robinet, tout doux.
-narrateur|L'eau est tiède.
-narrateur|Elle brille sur les carreaux.
-enfant-m|Je n'atteins pas.
-maman|Sarah tient le camion.
-maman|Toi, tu frottes les roues.
-maman|Vous jouez ensemble.
-maman|On peut jouer ensemble.
-narrateur|Sarah tient le toit sous l'eau.
-narrateur|Amir frotte les roues.
-narrateur|Le torchon est mouillé, maintenant.
-enfant-m|Ça mousse un peu !
-maman|Oui.
-copine|Le toit brille.
-enfant-m|Les roues aussi.
-narrateur|Une goutte tombe sur un carreau.
-narrateur|Elle fait un petit chemin.
-maman|On laisse la coccinelle ?
+narrateur|Sarah pose une main sur le toit.
+narrateur|Amir pose une main sur une roue.
+enfant-f|Moi, je mets de l'eau.
+enfant-m|Moi, les roues.
+papa|Un peu d'eau ?
+enfant-m|Oui, papa.
+narrateur|Un filet tiède tombe sur la pierre.
+narrateur|Amir tire vers les roues.
+narrateur|Sarah tire vers l'eau.
+enfant-m|Les roues, Sarah !
+enfant-f|L'eau d'abord !
+narrateur|Le camion glisse.
+narrateur|Il tape la pierre.
+narrateur|L'eau gicle sur le torchon.
+enfant-m|Oh.
+enfant-f|Il est parti.
+narrateur|L'éclat de robinet saute.
+narrateur|Une goutte le cache.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux le camion propre ?
+enfant-m|Oui, papa.
+maman|Sarah, tu le tiens ?
+enfant-f|Oui, maman.
+papa|Tu tiens ma manche, Amir ?
 enfant-m|Oui.
-narrateur|Le camion n'a plus de poussière.
-narrateur|Le bois est foncé, tout propre.
-narrateur|Une goutte reste sur le capot.
-enfant-m|Elle brille.
-maman|Oui.
-maman|Le bois a bu un peu.</t>
+narrateur|Amir veut recommencer tout de suite.
+narrateur|Ses doigts foncent vers le bois.
+enfant-m|Je le veux maintenant !</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>robinet,goutte,camion</t>
         </is>
       </c>
     </row>
@@ -1407,12 +1425,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Amir invite Sarah. Que font-ils ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Amir invite &lt;emphasis level="moderate"&gt;Sarah&lt;/emphasis&gt;. Que font-ils ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Achille invite Diane. Que font-ils ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Amir invite &lt;emphasis&gt;Sarah&lt;/emphasis&gt;. Que font-ils ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1475,7 +1493,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1483,10 +1501,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1501,34 +1519,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Sarah</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1537,13 +1559,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1553,7 +1575,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=amir_invite_sarah_ils_jouent; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1586,17 +1608,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir essuie une roue. Sarah essuie le toit. Les deux façons marchent. Il est lisse, maintenant. Oui. Vous avez des tailles différentes. Et vous jouez ensemble. Ils tapent des mains, tout doux. Le torchon goutte sur la pierre. On fait le voyage ? Oui. Un plaid attend près des tomates. Il sent le soleil. Amir pousse le camion. Sarah marche à côté. Les roues font un bruit mouillé. Il va au garage. Le plaid est le garage ? Oui, maman. La coccinelle est encore là. Les carreaux sèchent déjà. Le camion a bien voyagé ? Oui.</t>
+          <t>Amir ouvre les mains trop vite. Il veut tirer le camion, seul. Le bois glisse de nouveau. Oh. Le sourire ne revient pas. Amir refuse de foncer. Sarah s'arrête aussi. Personne ne dit la suite. Ils écoutent le tic du robinet. Une goutte glisse sur le métal. L'éclat de robinet revient. Il est là, Sarah. Je le vois. Tu le vois sur le bec ? Oui, papa. Le torchon, près de la pierre ? Je le prends. Sarah tient le toit, plus haut. Amir n'atteint pas le bec. C'est haut. Je tiens. Un filet, juste un peu ? Oui. L'eau tiède touche le toit. Amir frotte les roues, plus bas. Le torchon à carreaux devient mouillé. Ça mousse un peu ! Le toit brille. Les roues aussi. Le bois a bu un peu ? Oui, maman. Merci, Amir. Papa a regardé jusqu'au bout. On fait le voyage ? Oui. Un plaid attend près des tomates. Il sent le soleil. Le plaid est le garage ? Oui, papa. Sarah, tu marches à côté ? Oui, maman. Sarah garde une main sur le toit. Amir pousse une roue, lente.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir essuie une roue. Sarah essuie le toit. Les deux façons marchent. Il est lisse, maintenant. Oui. Vous avez des tailles différentes. Et vous jouez ensemble. Ils tapent des mains, tout doux. Le torchon goutte sur la pierre. On fait le voyage ? Oui. Un plaid attend près des tomates. Il sent le soleil. Amir pousse le camion. Sarah marche à côté. Les roues font un bruit mouillé. Il va au garage. Le plaid est le garage ? Oui, maman. La coccinelle est encore là. Les carreaux sèchent déjà. Le camion a bien voyagé ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir ouvre les mains trop vite. Il veut tirer le camion, seul. Le bois glisse de nouveau. Oh. Le sourire ne revient pas. Amir refuse de foncer. Sarah s'arrête aussi. Personne ne dit la suite. Ils écoutent le tic du robinet. Une goutte glisse sur le métal. L'&lt;emphasis level="moderate"&gt;éclat de robinet&lt;/emphasis&gt; revient. Il est là, Sarah. Je le vois. Tu le vois sur le bec ? Oui, papa. Le torchon, près de la pierre ? Je le prends. Sarah tient le toit, plus haut. Amir n'atteint pas le bec. C'est haut. Je tiens. Un filet, juste un peu ? Oui. L'eau tiède touche le toit. Amir frotte les roues, plus bas. Le torchon à carreaux devient mouillé. Ça mousse un peu ! Le toit brille. Les roues aussi. Le bois a bu un peu ? Oui, maman. Merci, Amir. Papa a regardé jusqu'au bout. On fait le voyage ? Oui. Un plaid attend près des tomates. Il sent le soleil. Le plaid est le garage ? Oui, papa. Sarah, tu marches à côté ? Oui, maman. Sarah garde une main sur le toit. Amir pousse une roue, lente.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Achille a invité. Diane a dit oui. Ils ont des &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. Ils jouent ensemble.&lt;/slow&gt; [pause]</t>
+          <t>Amir ouvre les mains trop vite. Il veut tirer le camion, seul. Le bois glisse de nouveau. Oh. Le sourire ne revient pas. Amir refuse de foncer. Sarah s'arrête aussi. Personne ne dit la suite. Ils écoutent le tic du robinet. Une goutte glisse sur le métal. L'&lt;emphasis&gt;éclat de robinet&lt;/emphasis&gt; revient. Il est là, Sarah. Je le vois. Tu le vois sur le bec ? Oui, papa. Le torchon, près de la pierre ? Je le prends. Sarah tient le toit, plus haut. Amir n'atteint pas le bec. C'est haut. Je tiens. Un filet, juste un peu ? Oui. L'eau tiède touche le toit. Amir frotte les roues, plus bas. Le torchon à carreaux devient mouillé. Ça mousse un peu ! Le toit brille. Les roues aussi. Le bois a bu un peu ? Oui, maman. Merci, Amir. Papa a regardé jusqu'au bout. On fait le voyage ? Oui. Un plaid attend près des tomates. Il sent le soleil. Le plaid est le garage ? Oui, papa. Sarah, tu marches à côté ? Oui, maman. Sarah garde une main sur le toit. Amir pousse une roue, lente. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1643,18 +1665,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1677,30 +1699,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>éclat de robinet</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1709,10 +1731,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,38 +1743,63 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=sarah_tient_le_toit_amir_frotte_les_roues; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir essuie une roue.
-narrateur|Sarah essuie le toit.
-narrateur|Les deux façons marchent.
-enfant-m|Il est lisse, maintenant.
-maman|Oui.
-maman|Vous avez des tailles différentes.
-maman|Et vous jouez ensemble.
-narrateur|Ils tapent des mains, tout doux.
-narrateur|Le torchon goutte sur la pierre.
-copine|On fait le voyage ?
+          <t>narrateur|Amir ouvre les mains trop vite.
+narrateur|Il veut tirer le camion, seul.
+narrateur|Le bois glisse de nouveau.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Amir refuse de foncer.
+narrateur|Sarah s'arrête aussi.
+narrateur|Personne ne dit la suite.
+narrateur|Ils écoutent le tic du robinet.
+narrateur|Une goutte glisse sur le métal.
+narrateur|L'éclat de robinet revient.
+enfant-m|Il est là, Sarah.
+enfant-f|Je le vois.
+papa|Tu le vois sur le bec ?
+enfant-m|Oui, papa.
+maman|Le torchon, près de la pierre ?
+enfant-f|Je le prends.
+narrateur|Sarah tient le toit, plus haut.
+narrateur|Amir n'atteint pas le bec.
+enfant-m|C'est haut.
+enfant-f|Je tiens.
+papa|Un filet, juste un peu ?
+enfant-f|Oui.
+narrateur|L'eau tiède touche le toit.
+narrateur|Amir frotte les roues, plus bas.
+narrateur|Le torchon à carreaux devient mouillé.
+enfant-m|Ça mousse un peu !
+enfant-f|Le toit brille.
+enfant-m|Les roues aussi.
+maman|Le bois a bu un peu ?
+enfant-m|Oui, maman.
+papa|Merci, Amir.
+narrateur|Papa a regardé jusqu'au bout.
+enfant-f|On fait le voyage ?
 enfant-m|Oui.
 narrateur|Un plaid attend près des tomates.
 narrateur|Il sent le soleil.
-narrateur|Amir pousse le camion.
-narrateur|Sarah marche à côté.
-narrateur|Les roues font un bruit mouillé.
-enfant-m|Il va au garage.
-maman|Le plaid est le garage ?
-enfant-m|Oui, maman.
-narrateur|La coccinelle est encore là.
-narrateur|Les carreaux sèchent déjà.
-maman|Le camion a bien voyagé ?
-enfant-m|Oui.</t>
+papa|Le plaid est le garage ?
+enfant-m|Oui, papa.
+maman|Sarah, tu marches à côté ?
+enfant-f|Oui, maman.
+narrateur|Sarah garde une main sur le toit.
+narrateur|Amir pousse une roue, lente.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>robinet,torchon</t>
         </is>
       </c>
     </row>
@@ -1779,17 +1826,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On pose le camion sur le plaid ? Oui. Amir pose le camion. Sarah pose le torchon. Le bois sèche au soleil. Tu as fini de poser le camion ? Oui, maman. À demain. À demain. Le robinet ne goutte plus. Les carreaux redeviennent calmes. Le plaid garde une petite trace d'eau.</t>
+          <t>Amir pousse le camion trop vite. Sarah marche trop loin, devant. Les roues font un bruit mouillé. Il va au garage ! Le camion part de travers. Le torchon tombe sur la pierre. Il file ! Amir veut le rattraper, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Toi un bord. Moi l'autre. Sarah se met d'un côté. Amir se met de l'autre. Ils poussent, sans se presser. Tes pieds sont près des roues ? Oui, papa. Sarah, tu tiens le toit ? Oui, maman. Le camion avance, droit. Il arrive sur le plaid. Le garage, Sarah. Il est chaud. Le plaid garde une petite trace d'eau. Le bois sèche au soleil ? Oui, maman. Le torchon, sur la pierre ? Je le pose. Sarah pose le torchon à carreaux. Amir pose le camion, deux mains.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On pose le camion sur le plaid ? Oui. Amir pose le camion. Sarah pose le torchon. Le bois sèche au soleil. Tu as fini de poser le camion ? Oui, maman. À demain. À demain. Le robinet ne goutte plus. Les carreaux redeviennent calmes. Le plaid garde une petite trace d'eau.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir pousse le &lt;emphasis level="moderate"&gt;camion&lt;/emphasis&gt; trop vite. Sarah marche trop loin, devant. Les roues font un bruit mouillé. Il va au garage ! Le camion part de travers. Le torchon tombe sur la pierre. Il file ! Amir veut le rattraper, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Toi un bord. Moi l'autre. Sarah se met d'un côté. Amir se met de l'autre. Ils poussent, sans se presser. Tes pieds sont près des roues ? Oui, papa. Sarah, tu tiens le toit ? Oui, maman. Le camion avance, droit. Il arrive sur le plaid. Le garage, Sarah. Il est chaud. Le plaid garde une petite trace d'eau. Le bois sèche au soleil ? Oui, maman. Le torchon, sur la pierre ? Je le pose. Sarah pose le torchon à carreaux. Amir pose le camion, deux mains.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Maman dit : on range. Achille range un seau. Diane range une pelle.&lt;/slow&gt; [pause]</t>
+          <t>Amir pousse le &lt;emphasis&gt;camion&lt;/emphasis&gt; trop vite. Sarah marche trop loin, devant. Les roues font un bruit mouillé. Il va au garage ! Le camion part de travers. Le torchon tombe sur la pierre. Il file ! Amir veut le rattraper, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Toi un bord. Moi l'autre. Sarah se met d'un côté. Amir se met de l'autre. Ils poussent, sans se presser. Tes pieds sont près des roues ? Oui, papa. Sarah, tu tiens le toit ? Oui, maman. Le camion avance, droit. Il arrive sur le plaid. Le garage, Sarah. Il est chaud. Le plaid garde une petite trace d'eau. Le bois sèche au soleil ? Oui, maman. Le torchon, sur la pierre ? Je le pose. Sarah pose le torchon à carreaux. Amir pose le camion, deux mains. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1836,18 +1883,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1868,28 +1915,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>camion</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1898,10 +1949,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1910,23 +1961,52 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=ils_prennent_le_camion_des_deux_bords; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On pose le camion sur le plaid ?
-enfant-m|Oui.
-narrateur|Amir pose le camion.
-narrateur|Sarah pose le torchon.
-narrateur|Le bois sèche au soleil.
-maman|Tu as fini de poser le camion ?
+          <t>narrateur|Amir pousse le camion trop vite.
+narrateur|Sarah marche trop loin, devant.
+narrateur|Les roues font un bruit mouillé.
+enfant-m|Il va au garage !
+narrateur|Le camion part de travers.
+narrateur|Le torchon tombe sur la pierre.
+enfant-f|Il file !
+narrateur|Amir veut le rattraper, d'un coup.
+narrateur|Amir refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|Personne ne dit la suite.
+enfant-f|Toi un bord.
+enfant-m|Moi l'autre.
+narrateur|Sarah se met d'un côté.
+narrateur|Amir se met de l'autre.
+narrateur|Ils poussent, sans se presser.
+papa|Tes pieds sont près des roues ?
+enfant-m|Oui, papa.
+maman|Sarah, tu tiens le toit ?
+enfant-f|Oui, maman.
+narrateur|Le camion avance, droit.
+narrateur|Il arrive sur le plaid.
+enfant-m|Le garage, Sarah.
+enfant-f|Il est chaud.
+narrateur|Le plaid garde une petite trace d'eau.
+maman|Le bois sèche au soleil ?
 enfant-m|Oui, maman.
-copine|À demain.
-enfant-m|À demain.
-narrateur|Le robinet ne goutte plus.
-narrateur|Les carreaux redeviennent calmes.
-narrateur|Le plaid garde une petite trace d'eau.</t>
+papa|Le torchon, sur la pierre ?
+enfant-f|Je le pose.
+narrateur|Sarah pose le torchon à carreaux.
+narrateur|Amir pose le camion, deux mains.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>camion,plaid</t>
         </is>
       </c>
     </row>
@@ -1953,17 +2033,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le camion est propre. On a joué ensemble. Bravo, Amir. Le torchon sèche encore.</t>
+          <t>Ils restent près du plaid. Le camion de bois repose, propre. L'éclat est là, papa. Tu le vois sur le bec ? Oui, papa. On est bien, ici. Le robinet fait tic, plus petit. Le torchon à carreaux sèche. Le toit est lisse. Les roues aussi. Amir pose la joue près du bois. Le bois est froid, un peu. C'est froid. Tu le sens sur tes joues ? Oui, il est froid. Il a voyagé. Jusqu'au plaid ? Oui, maman. Le capot porte une trace de paume. Dehors, le jardin s'endort. L'éclat de robinet tient sur le métal.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le camion est propre. On a joué ensemble. Bravo, Amir. Le torchon sèche encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du plaid. Le camion de bois repose, propre. L'éclat est là, papa. Tu le vois sur le bec ? Oui, papa. On est bien, ici. Le robinet fait tic, plus petit. Le torchon à carreaux sèche. Le toit est lisse. Les roues aussi. Amir pose la joue près du bois. Le bois est froid, un peu. C'est froid. Tu le sens sur tes joues ? Oui, il est froid. Il a voyagé. Jusqu'au plaid ? Oui, maman. Le capot porte une trace de paume. Dehors, le jardin s'endort. L'&lt;emphasis level="moderate"&gt;éclat de robinet&lt;/emphasis&gt; tient sur le métal.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du plaid. Le camion de bois repose, propre. L'éclat est là, papa. Tu le vois sur le bec ? Oui, papa. On est bien, ici. Le robinet fait tic, plus petit. Le torchon à carreaux sèche. Le toit est lisse. Les roues aussi. Amir pose la joue près du bois. Le bois est froid, un peu. C'est froid. Tu le sens sur tes joues ? Oui, il est froid. Il a voyagé. Jusqu'au plaid ? Oui, maman. Le capot porte une trace de paume. Dehors, le jardin s'endort. L'&lt;emphasis&gt;éclat de robinet&lt;/emphasis&gt; tient sur le métal.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2010,7 +2090,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2018,7 +2098,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2030,12 +2110,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2044,17 +2124,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de robinet</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2063,11 +2147,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2076,27 +2160,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_metal; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|Le camion est propre.
-enfant-m|On a joué ensemble.
-maman|Bravo, Amir.
-narrateur|Le torchon sèche encore.</t>
+          <t>narrateur|Ils restent près du plaid.
+narrateur|Le camion de bois repose, propre.
+enfant-m|L'éclat est là, papa.
+papa|Tu le vois sur le bec ?
+enfant-m|Oui, papa.
+maman|On est bien, ici.
+narrateur|Le robinet fait tic, plus petit.
+narrateur|Le torchon à carreaux sèche.
+enfant-f|Le toit est lisse.
+enfant-m|Les roues aussi.
+narrateur|Amir pose la joue près du bois.
+narrateur|Le bois est froid, un peu.
+enfant-m|C'est froid.
+papa|Tu le sens sur tes joues ?
+enfant-m|Oui, il est froid.
+enfant-f|Il a voyagé.
+maman|Jusqu'au plaid ?
+enfant-m|Oui, maman.
+narrateur|Le capot porte une trace de paume.
+narrateur|Dehors, le jardin s'endort.
+narrateur|L'éclat de robinet tient sur le métal.</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2195,6 +2300,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>